<commit_message>
Step 10.1: Autonomous queue and data export improvements
</commit_message>
<xml_diff>
--- a/Geocoded_Ad_Targeting_Locations_FINAL.xlsx
+++ b/Geocoded_Ad_Targeting_Locations_FINAL.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP\Documents\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP\Downloads\G-Map_Data_Scraper_2.0\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{00823F2F-84C3-43A6-8D63-00335598DCF7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D16D1C9B-C934-4208-AAC1-B635E25BE624}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{2EFE7CA6-FAD9-449D-9EE4-AAC15D71DE5D}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="295" uniqueCount="159">
   <si>
     <t>PIN Code</t>
   </si>
@@ -181,6 +181,327 @@
   </si>
   <si>
     <t>Longitude</t>
+  </si>
+  <si>
+    <t>District</t>
+  </si>
+  <si>
+    <t>State</t>
+  </si>
+  <si>
+    <t>Tehsil</t>
+  </si>
+  <si>
+    <t>AMROHA</t>
+  </si>
+  <si>
+    <t>Uttar Pradesh</t>
+  </si>
+  <si>
+    <t>Amroha</t>
+  </si>
+  <si>
+    <t>MORADABAD</t>
+  </si>
+  <si>
+    <t>Kanth</t>
+  </si>
+  <si>
+    <t>Thakurdwara</t>
+  </si>
+  <si>
+    <t>DEORIA</t>
+  </si>
+  <si>
+    <t>Deoria</t>
+  </si>
+  <si>
+    <t>GORAKHPUR</t>
+  </si>
+  <si>
+    <t>Chauri Chaura</t>
+  </si>
+  <si>
+    <t>Gorakhpur</t>
+  </si>
+  <si>
+    <t>Khajni</t>
+  </si>
+  <si>
+    <t>JAIPUR</t>
+  </si>
+  <si>
+    <t>Rajasthan</t>
+  </si>
+  <si>
+    <t>Mauzamabad</t>
+  </si>
+  <si>
+    <t>LUCKNOW</t>
+  </si>
+  <si>
+    <t>Bakshi Ka Talab</t>
+  </si>
+  <si>
+    <t>Sadar</t>
+  </si>
+  <si>
+    <t>SITAPUR</t>
+  </si>
+  <si>
+    <t>Laharpur</t>
+  </si>
+  <si>
+    <t>DHULE</t>
+  </si>
+  <si>
+    <t>Maharashtra</t>
+  </si>
+  <si>
+    <t>Dhule</t>
+  </si>
+  <si>
+    <t>Sakri</t>
+  </si>
+  <si>
+    <t>Sindkhede</t>
+  </si>
+  <si>
+    <t>NASHIK</t>
+  </si>
+  <si>
+    <t>Baglan</t>
+  </si>
+  <si>
+    <t>Nandgaon</t>
+  </si>
+  <si>
+    <t>Surgana</t>
+  </si>
+  <si>
+    <t>Yevla</t>
+  </si>
+  <si>
+    <t>THANE</t>
+  </si>
+  <si>
+    <t>Ambarnath</t>
+  </si>
+  <si>
+    <t>Kalyan</t>
+  </si>
+  <si>
+    <t>AMBALA</t>
+  </si>
+  <si>
+    <t>Haryana</t>
+  </si>
+  <si>
+    <t>Barara</t>
+  </si>
+  <si>
+    <t>BHIWANI</t>
+  </si>
+  <si>
+    <t>Bawani Khera</t>
+  </si>
+  <si>
+    <t>Bhiwani</t>
+  </si>
+  <si>
+    <t>FATEHABAD</t>
+  </si>
+  <si>
+    <t>Fatehabad</t>
+  </si>
+  <si>
+    <t>Ratia</t>
+  </si>
+  <si>
+    <t>Tohana</t>
+  </si>
+  <si>
+    <t>FAZILKA</t>
+  </si>
+  <si>
+    <t>Punjab</t>
+  </si>
+  <si>
+    <t>Abohar</t>
+  </si>
+  <si>
+    <t>Fazilka</t>
+  </si>
+  <si>
+    <t>GURDASPUR</t>
+  </si>
+  <si>
+    <t>Batala</t>
+  </si>
+  <si>
+    <t>Dera Baba Nanak</t>
+  </si>
+  <si>
+    <t>Gurdaspur</t>
+  </si>
+  <si>
+    <t>HOSHIARPUR</t>
+  </si>
+  <si>
+    <t>Garhshankar</t>
+  </si>
+  <si>
+    <t>Hoshiarpur</t>
+  </si>
+  <si>
+    <t>JALANDHAR</t>
+  </si>
+  <si>
+    <t>Jalandhar - I</t>
+  </si>
+  <si>
+    <t>Jalandhar - II</t>
+  </si>
+  <si>
+    <t>Phillaur</t>
+  </si>
+  <si>
+    <t>KARNAL</t>
+  </si>
+  <si>
+    <t>Indri</t>
+  </si>
+  <si>
+    <t>Karnal</t>
+  </si>
+  <si>
+    <t>Nilokheri</t>
+  </si>
+  <si>
+    <t>LUDHIANA</t>
+  </si>
+  <si>
+    <t>Jagraon</t>
+  </si>
+  <si>
+    <t>Ludhiana (East)</t>
+  </si>
+  <si>
+    <t>Ludhiana (West)</t>
+  </si>
+  <si>
+    <t>Samrala</t>
+  </si>
+  <si>
+    <t>SIRSA</t>
+  </si>
+  <si>
+    <t>Dabwali</t>
+  </si>
+  <si>
+    <t>Ellenabad</t>
+  </si>
+  <si>
+    <t>Rania</t>
+  </si>
+  <si>
+    <t>Sirsa</t>
+  </si>
+  <si>
+    <t>YAMUNANAGAR</t>
+  </si>
+  <si>
+    <t>Bilaspur</t>
+  </si>
+  <si>
+    <t>Chhachhrauli</t>
+  </si>
+  <si>
+    <t>Jagadhri</t>
+  </si>
+  <si>
+    <t>Anchor Village/Town</t>
+  </si>
+  <si>
+    <t>Buderna (HQ/Town - CSP location, not a distinct rural village)</t>
+  </si>
+  <si>
+    <t>Serua Dharmpur (HQ/Town - CSP location, not a distinct rural village)</t>
+  </si>
+  <si>
+    <t>Sihali Khaddar</t>
+  </si>
+  <si>
+    <t>Khairatia</t>
+  </si>
+  <si>
+    <t>Saraiya</t>
+  </si>
+  <si>
+    <t>Arazi Chauri</t>
+  </si>
+  <si>
+    <t>Baghari</t>
+  </si>
+  <si>
+    <t>Bharasi</t>
+  </si>
+  <si>
+    <t>Dheku Nadh</t>
+  </si>
+  <si>
+    <t>Karimnagar</t>
+  </si>
+  <si>
+    <t>Shiv Nagar Rooppur Khadra (HQ/Town - CSP location, not a distinct rural village)</t>
+  </si>
+  <si>
+    <t>Badauntola (HQ/Town - CSP location, not a distinct rural village)</t>
+  </si>
+  <si>
+    <t>Navi Nagar</t>
+  </si>
+  <si>
+    <t>Rangwa</t>
+  </si>
+  <si>
+    <t>Ambode</t>
+  </si>
+  <si>
+    <t>Nikumbhe</t>
+  </si>
+  <si>
+    <t>Chhadwel (p)</t>
+  </si>
+  <si>
+    <t>Khudane</t>
+  </si>
+  <si>
+    <t>Sukapur</t>
+  </si>
+  <si>
+    <t>Daul</t>
+  </si>
+  <si>
+    <t>Nampur</t>
+  </si>
+  <si>
+    <t>Mandwad</t>
+  </si>
+  <si>
+    <t>Jaykheda (HQ/Town - CSP location, not a distinct rural village)</t>
+  </si>
+  <si>
+    <t>Babhulgaon Bk.</t>
+  </si>
+  <si>
+    <t>Yeola (HQ/Town - CSP location, not a distinct rural village)</t>
+  </si>
+  <si>
+    <t>Ulhasnagar (HQ/Town - CSP location, not a distinct rural village)</t>
+  </si>
+  <si>
+    <t>Khadavali</t>
   </si>
 </sst>
 </file>
@@ -255,7 +576,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -263,29 +584,29 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -293,11 +614,160 @@
     <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="1">
+  <dxfs count="8">
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -306,6 +776,45 @@
         </patternFill>
       </fill>
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="0"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="4" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -321,12 +830,16 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{40D995E3-44C6-468A-840D-F24E2D0786F7}" name="Table1" displayName="Table1" ref="A1:C59" totalsRowShown="0">
-  <autoFilter ref="A1:C59" xr:uid="{40D995E3-44C6-468A-840D-F24E2D0786F7}"/>
-  <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{6667905F-B31C-47BA-93E7-8506475DE500}" name="PIN Code" dataDxfId="0"/>
-    <tableColumn id="2" xr3:uid="{755243FA-4E53-40DE-B529-B2791CD1B1FD}" name="Latitude"/>
-    <tableColumn id="3" xr3:uid="{55A18A85-46A1-495A-9440-205C59ADC104}" name="Longitude"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{40D995E3-44C6-468A-840D-F24E2D0786F7}" name="Table1" displayName="Table1" ref="A1:G59" totalsRowShown="0" headerRowDxfId="7">
+  <autoFilter ref="A1:G59" xr:uid="{40D995E3-44C6-468A-840D-F24E2D0786F7}"/>
+  <tableColumns count="7">
+    <tableColumn id="1" xr3:uid="{6667905F-B31C-47BA-93E7-8506475DE500}" name="PIN Code" dataDxfId="6"/>
+    <tableColumn id="2" xr3:uid="{755243FA-4E53-40DE-B529-B2791CD1B1FD}" name="Latitude" dataDxfId="5"/>
+    <tableColumn id="3" xr3:uid="{55A18A85-46A1-495A-9440-205C59ADC104}" name="Longitude" dataDxfId="4"/>
+    <tableColumn id="4" xr3:uid="{C3D71773-A2D3-4CC0-8BC2-8695E2B3163C}" name="District" dataDxfId="3"/>
+    <tableColumn id="5" xr3:uid="{25964E71-531A-4D40-BAEB-BA3A40B09B59}" name="State" dataDxfId="2"/>
+    <tableColumn id="6" xr3:uid="{1AFA86D0-4F46-498B-89E3-98F451B87AE7}" name="Tehsil" dataDxfId="1"/>
+    <tableColumn id="7" xr3:uid="{35C09263-657F-45F6-BF77-1A2A05F66854}" name="Anchor Village/Town" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -629,27 +1142,43 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6B92FE42-A60B-4A3F-BBB0-B7F38A1791FE}">
-  <dimension ref="A1:C59"/>
+  <dimension ref="A1:G59"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="15.36328125" style="5" customWidth="1"/>
+    <col min="1" max="1" width="15.36328125" style="1" customWidth="1"/>
     <col min="2" max="2" width="17.08984375" customWidth="1"/>
     <col min="3" max="3" width="19.26953125" customWidth="1"/>
+    <col min="4" max="4" width="15.7265625" customWidth="1"/>
+    <col min="5" max="5" width="14.81640625" customWidth="1"/>
+    <col min="6" max="6" width="27.7265625" customWidth="1"/>
+    <col min="7" max="7" width="70.6328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A1" s="7" t="s">
+    <row r="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="8" t="s">
+      <c r="B1" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="C1" s="8" t="s">
+      <c r="C1" s="3" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A2" s="1" t="s">
+      <c r="D1" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="F1" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="G1" s="4" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A2" s="5" t="s">
         <v>1</v>
       </c>
       <c r="B2" s="6">
@@ -658,632 +1187,1328 @@
       <c r="C2" s="6">
         <v>78.474427199999994</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A3" s="2" t="s">
+      <c r="D2" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="E2" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="F2" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="G2" s="7" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A3" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="B3">
+      <c r="B3" s="7">
         <v>29.006396500000001</v>
       </c>
-      <c r="C3">
+      <c r="C3" s="7">
         <v>78.703469200000001</v>
       </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A4" s="2" t="s">
+      <c r="D3" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="E3" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="F3" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="G3" s="7" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A4" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="B4">
+      <c r="B4" s="7">
         <v>29.004349600000001</v>
       </c>
-      <c r="C4">
+      <c r="C4" s="7">
         <v>78.746953000000005</v>
       </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A5" s="1" t="s">
+      <c r="D4" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="E4" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="F4" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="G4" s="7" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A5" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="B5">
+      <c r="B5" s="7">
         <v>26.666667</v>
       </c>
-      <c r="C5">
+      <c r="C5" s="7">
         <v>83.75</v>
       </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A6" s="1" t="s">
+      <c r="D5" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="E5" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="F5" s="7" t="s">
+        <v>62</v>
+      </c>
+      <c r="G5" s="7" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A6" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="B6">
+      <c r="B6" s="7">
         <v>26.6819089</v>
       </c>
-      <c r="C6">
+      <c r="C6" s="7">
         <v>83.570484800000003</v>
       </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A7" s="1">
+      <c r="D6" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="E6" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="F6" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="G6" s="7" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A7" s="5">
         <v>273001</v>
       </c>
-      <c r="B7">
+      <c r="B7" s="7">
         <v>26.760021699999999</v>
       </c>
-      <c r="C7">
+      <c r="C7" s="7">
         <v>83.366812899999999</v>
       </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A8" s="1" t="s">
+      <c r="D7" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="E7" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="F7" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="G7" s="7" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A8" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="B8">
+      <c r="B8" s="7">
         <v>26.760021699999999</v>
       </c>
-      <c r="C8">
+      <c r="C8" s="7">
         <v>83.366812899999999</v>
       </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A9" s="1" t="s">
+      <c r="D8" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="E8" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="F8" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="G8" s="7" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A9" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="B9">
+      <c r="B9" s="7">
         <v>26.552692</v>
       </c>
-      <c r="C9">
+      <c r="C9" s="7">
         <v>83.227005300000002</v>
       </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A10" s="1">
+      <c r="D9" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="E9" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="F9" s="7" t="s">
+        <v>66</v>
+      </c>
+      <c r="G9" s="7" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A10" s="5">
         <v>273213</v>
       </c>
-      <c r="B10">
+      <c r="B10" s="7">
         <v>26.552692</v>
       </c>
-      <c r="C10">
+      <c r="C10" s="7">
         <v>83.227005300000002</v>
       </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A11" s="1" t="s">
+      <c r="D10" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="E10" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="F10" s="7" t="s">
+        <v>66</v>
+      </c>
+      <c r="G10" s="7" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A11" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="B11">
+      <c r="B11" s="7">
         <v>26.672042900000001</v>
       </c>
-      <c r="C11">
+      <c r="C11" s="7">
         <v>75.361575999999999</v>
       </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A12" s="1" t="s">
+      <c r="D11" s="7" t="s">
+        <v>67</v>
+      </c>
+      <c r="E11" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="F11" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="G11" s="7" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A12" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="B12">
+      <c r="B12" s="7">
         <v>27.034942699999998</v>
       </c>
-      <c r="C12">
+      <c r="C12" s="7">
         <v>80.921437299999994</v>
       </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A13" s="1" t="s">
+      <c r="D12" s="7" t="s">
+        <v>70</v>
+      </c>
+      <c r="E12" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="F12" s="7" t="s">
+        <v>71</v>
+      </c>
+      <c r="G12" s="7" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A13" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="B13">
+      <c r="B13" s="7">
         <v>26.838100000000001</v>
       </c>
-      <c r="C13">
+      <c r="C13" s="7">
         <v>80.934600099999997</v>
       </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A14" s="2" t="s">
+      <c r="D13" s="7" t="s">
+        <v>70</v>
+      </c>
+      <c r="E13" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="F13" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="G13" s="7" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A14" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="B14">
+      <c r="B14" s="7">
         <v>27.725634500000002</v>
       </c>
-      <c r="C14">
+      <c r="C14" s="7">
         <v>80.986922300000003</v>
       </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A15" s="2" t="s">
+      <c r="D14" s="7" t="s">
+        <v>73</v>
+      </c>
+      <c r="E14" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="F14" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="G14" s="7" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A15" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="B15">
+      <c r="B15" s="7">
         <v>27.725634500000002</v>
       </c>
-      <c r="C15">
+      <c r="C15" s="7">
         <v>80.986922300000003</v>
       </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A16" s="2" t="s">
+      <c r="D15" s="7" t="s">
+        <v>73</v>
+      </c>
+      <c r="E15" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="F15" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="G15" s="7" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A16" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="B16">
+      <c r="B16" s="7">
         <v>27.725634500000002</v>
       </c>
-      <c r="C16">
+      <c r="C16" s="7">
         <v>80.986922300000003</v>
       </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A17" s="1" t="s">
+      <c r="D16" s="7" t="s">
+        <v>73</v>
+      </c>
+      <c r="E16" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="F16" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="G16" s="7" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A17" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="B17">
+      <c r="B17" s="7">
         <v>20.911056899999998</v>
       </c>
-      <c r="C17">
+      <c r="C17" s="7">
         <v>74.898519500000006</v>
       </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A18" s="3" t="s">
+      <c r="D17" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="E17" s="7" t="s">
+        <v>76</v>
+      </c>
+      <c r="F17" s="7" t="s">
+        <v>77</v>
+      </c>
+      <c r="G17" s="7" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A18" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="B18">
+      <c r="B18" s="7">
         <v>21.0516468</v>
       </c>
-      <c r="C18">
+      <c r="C18" s="7">
         <v>74.652442899999997</v>
       </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A19" s="3" t="s">
+      <c r="D18" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="E18" s="7" t="s">
+        <v>76</v>
+      </c>
+      <c r="F18" s="7" t="s">
+        <v>77</v>
+      </c>
+      <c r="G18" s="7" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A19" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="B19">
+      <c r="B19" s="7">
         <v>21.205897400000001</v>
       </c>
-      <c r="C19">
+      <c r="C19" s="7">
         <v>74.247117500000002</v>
       </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A20" s="3" t="s">
+      <c r="D19" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="E19" s="7" t="s">
+        <v>76</v>
+      </c>
+      <c r="F19" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="G19" s="7" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A20" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="B20">
+      <c r="B20" s="7">
         <v>21.1064507</v>
       </c>
-      <c r="C20">
+      <c r="C20" s="7">
         <v>74.285612</v>
       </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A21" s="1" t="s">
+      <c r="D20" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="E20" s="7" t="s">
+        <v>76</v>
+      </c>
+      <c r="F20" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="G20" s="7" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A21" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="B21">
+      <c r="B21" s="7">
         <v>20.923964600000001</v>
       </c>
-      <c r="C21">
+      <c r="C21" s="7">
         <v>74.078021000000007</v>
       </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A22" s="1" t="s">
+      <c r="D21" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="E21" s="7" t="s">
+        <v>76</v>
+      </c>
+      <c r="F21" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="G21" s="7" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A22" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="B22">
+      <c r="B22" s="7">
         <v>21.357449800000001</v>
       </c>
-      <c r="C22">
+      <c r="C22" s="7">
         <v>74.582593500000002</v>
       </c>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A23" s="4" t="s">
+      <c r="D22" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="E22" s="7" t="s">
+        <v>76</v>
+      </c>
+      <c r="F22" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="G22" s="7" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A23" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="B23">
+      <c r="B23" s="7">
         <v>20.729545699999999</v>
       </c>
-      <c r="C23">
+      <c r="C23" s="7">
         <v>74.310902400000003</v>
       </c>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A24" s="1" t="s">
+      <c r="D23" s="7" t="s">
+        <v>80</v>
+      </c>
+      <c r="E23" s="7" t="s">
+        <v>76</v>
+      </c>
+      <c r="F23" s="7" t="s">
+        <v>81</v>
+      </c>
+      <c r="G23" s="7" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A24" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="B24">
+      <c r="B24" s="7">
         <v>20.3094018</v>
       </c>
-      <c r="C24">
+      <c r="C24" s="7">
         <v>74.659762200000003</v>
       </c>
-    </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A25" s="1" t="s">
+      <c r="D24" s="7" t="s">
+        <v>80</v>
+      </c>
+      <c r="E24" s="7" t="s">
+        <v>76</v>
+      </c>
+      <c r="F24" s="7" t="s">
+        <v>82</v>
+      </c>
+      <c r="G24" s="7" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A25" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="B25">
+      <c r="B25" s="7">
         <v>20.559243200000001</v>
       </c>
-      <c r="C25">
+      <c r="C25" s="7">
         <v>73.637561399999996</v>
       </c>
-    </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A26" s="1" t="s">
+      <c r="D25" s="7" t="s">
+        <v>80</v>
+      </c>
+      <c r="E25" s="7" t="s">
+        <v>76</v>
+      </c>
+      <c r="F25" s="7" t="s">
+        <v>83</v>
+      </c>
+      <c r="G25" s="7" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A26" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="B26">
+      <c r="B26" s="7">
         <v>20.0112475</v>
       </c>
-      <c r="C26">
+      <c r="C26" s="7">
         <v>73.790236399999998</v>
       </c>
-    </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A27" s="1" t="s">
+      <c r="D26" s="7" t="s">
+        <v>80</v>
+      </c>
+      <c r="E26" s="7" t="s">
+        <v>76</v>
+      </c>
+      <c r="F26" s="7" t="s">
+        <v>84</v>
+      </c>
+      <c r="G26" s="7" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A27" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="B27">
+      <c r="B27" s="7">
         <v>20.036798000000001</v>
       </c>
-      <c r="C27">
+      <c r="C27" s="7">
         <v>74.486987999999997</v>
       </c>
-    </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A28" s="1" t="s">
+      <c r="D27" s="7" t="s">
+        <v>80</v>
+      </c>
+      <c r="E27" s="7" t="s">
+        <v>76</v>
+      </c>
+      <c r="F27" s="7" t="s">
+        <v>84</v>
+      </c>
+      <c r="G27" s="7" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A28" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="B28">
+      <c r="B28" s="7">
         <v>19.208879</v>
       </c>
-      <c r="C28">
+      <c r="C28" s="7">
         <v>73.152750999999995</v>
       </c>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A29" s="1" t="s">
+      <c r="D28" s="7" t="s">
+        <v>85</v>
+      </c>
+      <c r="E28" s="7" t="s">
+        <v>76</v>
+      </c>
+      <c r="F28" s="7" t="s">
+        <v>86</v>
+      </c>
+      <c r="G28" s="7" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A29" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="B29">
+      <c r="B29" s="7">
         <v>19.356724</v>
       </c>
-      <c r="C29">
+      <c r="C29" s="7">
         <v>73.219037499999999</v>
       </c>
-    </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A30" s="1" t="s">
+      <c r="D29" s="7" t="s">
+        <v>85</v>
+      </c>
+      <c r="E29" s="7" t="s">
+        <v>76</v>
+      </c>
+      <c r="F29" s="7" t="s">
+        <v>87</v>
+      </c>
+      <c r="G29" s="7" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A30" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="B30">
+      <c r="B30" s="7">
         <v>30.214222800000002</v>
       </c>
-      <c r="C30">
+      <c r="C30" s="7">
         <v>77.038364400000006</v>
       </c>
-    </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A31" s="1" t="s">
+      <c r="D30" s="7" t="s">
+        <v>88</v>
+      </c>
+      <c r="E30" s="7" t="s">
+        <v>89</v>
+      </c>
+      <c r="F30" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="G30" s="7" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A31" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="B31">
+      <c r="B31" s="7">
         <v>28.9497708</v>
       </c>
-      <c r="C31">
+      <c r="C31" s="7">
         <v>76.031748199999996</v>
       </c>
-    </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A32" s="1" t="s">
+      <c r="D31" s="7" t="s">
+        <v>91</v>
+      </c>
+      <c r="E31" s="7" t="s">
+        <v>89</v>
+      </c>
+      <c r="F31" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="G31" s="7" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A32" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="B32">
+      <c r="B32" s="7">
         <v>28.7931703</v>
       </c>
-      <c r="C32">
+      <c r="C32" s="7">
         <v>76.139128299999996</v>
       </c>
-    </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A33" s="1" t="s">
+      <c r="D32" s="7" t="s">
+        <v>91</v>
+      </c>
+      <c r="E32" s="7" t="s">
+        <v>89</v>
+      </c>
+      <c r="F32" s="7" t="s">
+        <v>93</v>
+      </c>
+      <c r="G32" s="7" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A33" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="B33">
+      <c r="B33" s="7">
         <v>29.511810799999999</v>
       </c>
-      <c r="C33">
+      <c r="C33" s="7">
         <v>75.429416399999994</v>
       </c>
-    </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A34" s="1" t="s">
+      <c r="D33" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="E33" s="7" t="s">
+        <v>89</v>
+      </c>
+      <c r="F33" s="7" t="s">
+        <v>95</v>
+      </c>
+      <c r="G33" s="7" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A34" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="B34">
+      <c r="B34" s="7">
         <v>29.686230699999999</v>
       </c>
-      <c r="C34">
+      <c r="C34" s="7">
         <v>75.575052099999994</v>
       </c>
-    </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A35" s="2" t="s">
+      <c r="D34" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="E34" s="7" t="s">
+        <v>89</v>
+      </c>
+      <c r="F34" s="7" t="s">
+        <v>96</v>
+      </c>
+      <c r="G34" s="7" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A35" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="B35">
+      <c r="B35" s="7">
         <v>29.7107922</v>
       </c>
-      <c r="C35">
+      <c r="C35" s="7">
         <v>75.9042326</v>
       </c>
-    </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A36" s="1" t="s">
+      <c r="D35" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="E35" s="7" t="s">
+        <v>89</v>
+      </c>
+      <c r="F35" s="7" t="s">
+        <v>97</v>
+      </c>
+      <c r="G35" s="7" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A36" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="B36">
+      <c r="B36" s="7">
         <v>30.139301499999998</v>
       </c>
-      <c r="C36">
+      <c r="C36" s="7">
         <v>74.194708500000004</v>
       </c>
-    </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A37" s="1" t="s">
+      <c r="D36" s="7" t="s">
+        <v>98</v>
+      </c>
+      <c r="E36" s="7" t="s">
+        <v>99</v>
+      </c>
+      <c r="F36" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="G36" s="7" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A37" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="B37">
+      <c r="B37" s="7">
         <v>30.403209700000001</v>
       </c>
-      <c r="C37">
+      <c r="C37" s="7">
         <v>74.0310609</v>
       </c>
-    </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A38" s="1" t="s">
+      <c r="D37" s="7" t="s">
+        <v>98</v>
+      </c>
+      <c r="E37" s="7" t="s">
+        <v>99</v>
+      </c>
+      <c r="F37" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="G37" s="7" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A38" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="B38">
+      <c r="B38" s="7">
         <v>31.819302499999999</v>
       </c>
-      <c r="C38">
+      <c r="C38" s="7">
         <v>75.199994099999998</v>
       </c>
-    </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A39" s="1" t="s">
+      <c r="D38" s="7" t="s">
+        <v>102</v>
+      </c>
+      <c r="E38" s="7" t="s">
+        <v>99</v>
+      </c>
+      <c r="F38" s="7" t="s">
+        <v>103</v>
+      </c>
+      <c r="G38" s="7" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A39" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="B39">
+      <c r="B39" s="7">
         <v>32.0459861</v>
       </c>
-      <c r="C39">
+      <c r="C39" s="7">
         <v>75.025856899999994</v>
       </c>
-    </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A40" s="1" t="s">
+      <c r="D39" s="7" t="s">
+        <v>102</v>
+      </c>
+      <c r="E39" s="7" t="s">
+        <v>99</v>
+      </c>
+      <c r="F39" s="7" t="s">
+        <v>104</v>
+      </c>
+      <c r="G39" s="7" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A40" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="B40">
+      <c r="B40" s="7">
         <v>32.041913399999999</v>
       </c>
-      <c r="C40">
+      <c r="C40" s="7">
         <v>75.400167699999997</v>
       </c>
-    </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A41" s="1" t="s">
+      <c r="D40" s="7" t="s">
+        <v>102</v>
+      </c>
+      <c r="E40" s="7" t="s">
+        <v>99</v>
+      </c>
+      <c r="F40" s="7" t="s">
+        <v>105</v>
+      </c>
+      <c r="G40" s="7" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A41" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="B41">
+      <c r="B41" s="7">
         <v>31.2226651</v>
       </c>
-      <c r="C41">
+      <c r="C41" s="7">
         <v>76.137604499999995</v>
       </c>
-    </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A42" s="1" t="s">
+      <c r="D41" s="7" t="s">
+        <v>106</v>
+      </c>
+      <c r="E41" s="7" t="s">
+        <v>99</v>
+      </c>
+      <c r="F41" s="7" t="s">
+        <v>107</v>
+      </c>
+      <c r="G41" s="7" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A42" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="B42">
+      <c r="B42" s="7">
         <v>31.532852299999998</v>
       </c>
-      <c r="C42">
+      <c r="C42" s="7">
         <v>75.902548499999995</v>
       </c>
-    </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A43" s="1" t="s">
+      <c r="D42" s="7" t="s">
+        <v>106</v>
+      </c>
+      <c r="E42" s="7" t="s">
+        <v>99</v>
+      </c>
+      <c r="F42" s="7" t="s">
+        <v>108</v>
+      </c>
+      <c r="G42" s="7" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A43" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="B43">
+      <c r="B43" s="7">
         <v>31.332376199999999</v>
       </c>
-      <c r="C43">
+      <c r="C43" s="7">
         <v>75.576888999999994</v>
       </c>
-    </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A44" s="1" t="s">
+      <c r="D43" s="7" t="s">
+        <v>109</v>
+      </c>
+      <c r="E43" s="7" t="s">
+        <v>99</v>
+      </c>
+      <c r="F43" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="G43" s="7" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A44" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="B44">
+      <c r="B44" s="7">
         <v>31.545745799999999</v>
       </c>
-      <c r="C44">
+      <c r="C44" s="7">
         <v>75.640382900000006</v>
       </c>
-    </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A45" s="1" t="s">
+      <c r="D44" s="7" t="s">
+        <v>109</v>
+      </c>
+      <c r="E44" s="7" t="s">
+        <v>99</v>
+      </c>
+      <c r="F44" s="7" t="s">
+        <v>111</v>
+      </c>
+      <c r="G44" s="7" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A45" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="B45">
+      <c r="B45" s="7">
         <v>31.016873199999999</v>
       </c>
-      <c r="C45">
+      <c r="C45" s="7">
         <v>75.786101900000006</v>
       </c>
-    </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A46" s="1" t="s">
+      <c r="D45" s="7" t="s">
+        <v>109</v>
+      </c>
+      <c r="E45" s="7" t="s">
+        <v>99</v>
+      </c>
+      <c r="F45" s="7" t="s">
+        <v>112</v>
+      </c>
+      <c r="G45" s="7" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A46" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="B46">
+      <c r="B46" s="7">
         <v>29.878940799999999</v>
       </c>
-      <c r="C46">
+      <c r="C46" s="7">
         <v>77.0520633</v>
       </c>
-    </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A47" s="1" t="s">
+      <c r="D46" s="7" t="s">
+        <v>113</v>
+      </c>
+      <c r="E46" s="7" t="s">
+        <v>89</v>
+      </c>
+      <c r="F46" s="7" t="s">
+        <v>114</v>
+      </c>
+      <c r="G46" s="7" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A47" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="B47">
+      <c r="B47" s="7">
         <v>29.6951152</v>
       </c>
-      <c r="C47">
+      <c r="C47" s="7">
         <v>76.969829200000007</v>
       </c>
-    </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A48" s="1" t="s">
+      <c r="D47" s="7" t="s">
+        <v>113</v>
+      </c>
+      <c r="E47" s="7" t="s">
+        <v>89</v>
+      </c>
+      <c r="F47" s="7" t="s">
+        <v>115</v>
+      </c>
+      <c r="G47" s="7" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="48" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A48" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="B48">
+      <c r="B48" s="7">
         <v>29.839773699999999</v>
       </c>
-      <c r="C48">
+      <c r="C48" s="7">
         <v>76.931802599999997</v>
       </c>
-    </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A49" s="1" t="s">
+      <c r="D48" s="7" t="s">
+        <v>113</v>
+      </c>
+      <c r="E48" s="7" t="s">
+        <v>89</v>
+      </c>
+      <c r="F48" s="7" t="s">
+        <v>116</v>
+      </c>
+      <c r="G48" s="7" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="49" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A49" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="B49">
+      <c r="B49" s="7">
         <v>30.800753799999999</v>
       </c>
-      <c r="C49">
+      <c r="C49" s="7">
         <v>75.472496699999994</v>
       </c>
-    </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A50" s="1" t="s">
+      <c r="D49" s="7" t="s">
+        <v>117</v>
+      </c>
+      <c r="E49" s="7" t="s">
+        <v>99</v>
+      </c>
+      <c r="F49" s="7" t="s">
+        <v>118</v>
+      </c>
+      <c r="G49" s="7" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="50" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A50" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="B50">
+      <c r="B50" s="7">
         <v>30.907070099999999</v>
       </c>
-      <c r="C50">
+      <c r="C50" s="7">
         <v>75.860780500000004</v>
       </c>
-    </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A51" s="1" t="s">
+      <c r="D50" s="7" t="s">
+        <v>117</v>
+      </c>
+      <c r="E50" s="7" t="s">
+        <v>99</v>
+      </c>
+      <c r="F50" s="7" t="s">
+        <v>119</v>
+      </c>
+      <c r="G50" s="7" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="51" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A51" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="B51">
+      <c r="B51" s="7">
         <v>30.909015700000001</v>
       </c>
-      <c r="C51">
+      <c r="C51" s="7">
         <v>75.851601000000002</v>
       </c>
-    </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A52" s="1" t="s">
+      <c r="D51" s="7" t="s">
+        <v>117</v>
+      </c>
+      <c r="E51" s="7" t="s">
+        <v>99</v>
+      </c>
+      <c r="F51" s="7" t="s">
+        <v>120</v>
+      </c>
+      <c r="G51" s="7" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="52" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A52" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="B52">
+      <c r="B52" s="7">
         <v>30.825246</v>
       </c>
-      <c r="C52">
+      <c r="C52" s="7">
         <v>76.177547500000003</v>
       </c>
-    </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A53" s="1" t="s">
+      <c r="D52" s="7" t="s">
+        <v>117</v>
+      </c>
+      <c r="E52" s="7" t="s">
+        <v>99</v>
+      </c>
+      <c r="F52" s="7" t="s">
+        <v>121</v>
+      </c>
+      <c r="G52" s="7" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="53" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A53" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="B53">
+      <c r="B53" s="7">
         <v>29.9486566</v>
       </c>
-      <c r="C53">
+      <c r="C53" s="7">
         <v>74.737280900000002</v>
       </c>
-    </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A54" s="1" t="s">
+      <c r="D53" s="7" t="s">
+        <v>122</v>
+      </c>
+      <c r="E53" s="7" t="s">
+        <v>89</v>
+      </c>
+      <c r="F53" s="7" t="s">
+        <v>123</v>
+      </c>
+      <c r="G53" s="7" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="54" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A54" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="B54">
+      <c r="B54" s="7">
         <v>29.444108</v>
       </c>
-      <c r="C54">
+      <c r="C54" s="7">
         <v>74.657949900000006</v>
       </c>
-    </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A55" s="1" t="s">
+      <c r="D54" s="7" t="s">
+        <v>122</v>
+      </c>
+      <c r="E54" s="7" t="s">
+        <v>89</v>
+      </c>
+      <c r="F54" s="7" t="s">
+        <v>124</v>
+      </c>
+      <c r="G54" s="7" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="55" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A55" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="B55">
+      <c r="B55" s="7">
         <v>29.5240902</v>
       </c>
-      <c r="C55">
+      <c r="C55" s="7">
         <v>74.836932700000006</v>
       </c>
-    </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A56" s="1" t="s">
+      <c r="D55" s="7" t="s">
+        <v>122</v>
+      </c>
+      <c r="E55" s="7" t="s">
+        <v>89</v>
+      </c>
+      <c r="F55" s="7" t="s">
+        <v>125</v>
+      </c>
+      <c r="G55" s="7" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="56" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A56" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="B56">
+      <c r="B56" s="7">
         <v>29.5372849</v>
       </c>
-      <c r="C56">
+      <c r="C56" s="7">
         <v>75.037764899999999</v>
       </c>
-    </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A57" s="1" t="s">
+      <c r="D56" s="7" t="s">
+        <v>122</v>
+      </c>
+      <c r="E56" s="7" t="s">
+        <v>89</v>
+      </c>
+      <c r="F56" s="7" t="s">
+        <v>126</v>
+      </c>
+      <c r="G56" s="7" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="57" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A57" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="B57">
+      <c r="B57" s="7">
         <v>30.3042628</v>
       </c>
-      <c r="C57">
+      <c r="C57" s="7">
         <v>77.302725300000006</v>
       </c>
-    </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A58" s="1" t="s">
+      <c r="D57" s="7" t="s">
+        <v>127</v>
+      </c>
+      <c r="E57" s="7" t="s">
+        <v>89</v>
+      </c>
+      <c r="F57" s="7" t="s">
+        <v>128</v>
+      </c>
+      <c r="G57" s="7" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="58" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A58" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="B58">
+      <c r="B58" s="7">
         <v>30.245567999999999</v>
       </c>
-      <c r="C58">
+      <c r="C58" s="7">
         <v>77.359232399999996</v>
       </c>
-    </row>
-    <row r="59" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A59" s="1" t="s">
+      <c r="D58" s="7" t="s">
+        <v>127</v>
+      </c>
+      <c r="E58" s="7" t="s">
+        <v>89</v>
+      </c>
+      <c r="F58" s="7" t="s">
+        <v>129</v>
+      </c>
+      <c r="G58" s="7" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="59" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A59" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="B59">
+      <c r="B59" s="7">
         <v>30.117322000000001</v>
       </c>
-      <c r="C59">
+      <c r="C59" s="7">
         <v>77.287663699999996</v>
+      </c>
+      <c r="D59" s="7" t="s">
+        <v>127</v>
+      </c>
+      <c r="E59" s="7" t="s">
+        <v>89</v>
+      </c>
+      <c r="F59" s="7" t="s">
+        <v>130</v>
+      </c>
+      <c r="G59" s="7" t="s">
+        <v>130</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Refuse coordinates that land outside the state they claim
Loading a spreadsheet of Gujarat PIN codes, a bare six-digit Maps search put
385002 in the Caucasus and three Kheda codes in Lucknow. Nothing downstream
would have questioned those rows: the district and state beside them read
correctly, and only the coordinates were wrong, so every business discovered
under them would have carried Gujarat geography while coming from Uttar
Pradesh.

A looked-up point is now checked against its state's rectangle, falling back
to the country for a state not listed, and the row is removed rather than
kept when it fails. Coordinates the caller typed are left alone — those are
theirs to get right. The message says what to do instead, since the cause is
an ambiguous search rather than a bad PIN.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Geocoded_Ad_Targeting_Locations_FINAL.xlsx
+++ b/Geocoded_Ad_Targeting_Locations_FINAL.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP\Downloads\G-Map_Data_Scraper_2.0\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D16D1C9B-C934-4208-AAC1-B635E25BE624}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8FF92AC9-4AE1-422F-8976-13A7F4FF7345}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{2EFE7CA6-FAD9-449D-9EE4-AAC15D71DE5D}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="295" uniqueCount="159">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="507" uniqueCount="182">
   <si>
     <t>PIN Code</t>
   </si>
@@ -502,13 +502,82 @@
   </si>
   <si>
     <t>Khadavali</t>
+  </si>
+  <si>
+    <t>Banaskantha</t>
+  </si>
+  <si>
+    <t>Sabarkantha</t>
+  </si>
+  <si>
+    <t>Ahmedabad</t>
+  </si>
+  <si>
+    <t>Kheda</t>
+  </si>
+  <si>
+    <t>Vadodara</t>
+  </si>
+  <si>
+    <t>Panchmahal</t>
+  </si>
+  <si>
+    <t>Gujarat</t>
+  </si>
+  <si>
+    <t>Palanpur</t>
+  </si>
+  <si>
+    <t>Palanpur area</t>
+  </si>
+  <si>
+    <t>Himatnagar</t>
+  </si>
+  <si>
+    <t>Hadiol/Himatnagar area</t>
+  </si>
+  <si>
+    <t>Rajpur/Himatnagar area</t>
+  </si>
+  <si>
+    <t>Ahmedabad City</t>
+  </si>
+  <si>
+    <t>Naroda</t>
+  </si>
+  <si>
+    <t>Naroda vicinity</t>
+  </si>
+  <si>
+    <t>Nikol/Naroda vicinity</t>
+  </si>
+  <si>
+    <t>Vatva</t>
+  </si>
+  <si>
+    <t>Vatva area</t>
+  </si>
+  <si>
+    <t>Vatva/GIDC</t>
+  </si>
+  <si>
+    <t>Nadiad</t>
+  </si>
+  <si>
+    <t>Vadodara City</t>
+  </si>
+  <si>
+    <t>Godhra</t>
+  </si>
+  <si>
+    <t>Bhuravav/Godhra</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -530,6 +599,13 @@
       <color theme="0"/>
       <name val="Calibri"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="8">
@@ -576,7 +652,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -599,11 +675,24 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -631,6 +720,14 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -830,8 +927,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{40D995E3-44C6-468A-840D-F24E2D0786F7}" name="Table1" displayName="Table1" ref="A1:G59" totalsRowShown="0" headerRowDxfId="7">
-  <autoFilter ref="A1:G59" xr:uid="{40D995E3-44C6-468A-840D-F24E2D0786F7}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{40D995E3-44C6-468A-840D-F24E2D0786F7}" name="Table1" displayName="Table1" ref="A1:G112" totalsRowShown="0" headerRowDxfId="7">
+  <autoFilter ref="A1:G112" xr:uid="{40D995E3-44C6-468A-840D-F24E2D0786F7}"/>
   <tableColumns count="7">
     <tableColumn id="1" xr3:uid="{6667905F-B31C-47BA-93E7-8506475DE500}" name="PIN Code" dataDxfId="6"/>
     <tableColumn id="2" xr3:uid="{755243FA-4E53-40DE-B529-B2791CD1B1FD}" name="Latitude" dataDxfId="5"/>
@@ -1142,7 +1239,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6B92FE42-A60B-4A3F-BBB0-B7F38A1791FE}">
-  <dimension ref="A1:G59"/>
+  <dimension ref="A1:G112"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="15.36328125" style="1" customWidth="1"/>
@@ -2511,6 +2608,1013 @@
         <v>130</v>
       </c>
     </row>
+    <row r="60" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A60" s="12">
+        <v>385001</v>
+      </c>
+      <c r="B60" s="7"/>
+      <c r="C60" s="7"/>
+      <c r="D60" s="11" t="s">
+        <v>159</v>
+      </c>
+      <c r="E60" s="11" t="s">
+        <v>165</v>
+      </c>
+      <c r="F60" s="11" t="s">
+        <v>166</v>
+      </c>
+      <c r="G60" s="11" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="61" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A61" s="12">
+        <v>385002</v>
+      </c>
+      <c r="B61" s="7"/>
+      <c r="C61" s="7"/>
+      <c r="D61" s="11" t="s">
+        <v>159</v>
+      </c>
+      <c r="E61" s="11" t="s">
+        <v>165</v>
+      </c>
+      <c r="F61" s="11" t="s">
+        <v>166</v>
+      </c>
+      <c r="G61" s="11" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="62" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A62" s="12">
+        <v>385010</v>
+      </c>
+      <c r="B62" s="7"/>
+      <c r="C62" s="7"/>
+      <c r="D62" s="11" t="s">
+        <v>159</v>
+      </c>
+      <c r="E62" s="11" t="s">
+        <v>165</v>
+      </c>
+      <c r="F62" s="11" t="s">
+        <v>166</v>
+      </c>
+      <c r="G62" s="11" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="63" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A63" s="12">
+        <v>383001</v>
+      </c>
+      <c r="B63" s="7"/>
+      <c r="C63" s="7"/>
+      <c r="D63" s="11" t="s">
+        <v>160</v>
+      </c>
+      <c r="E63" s="11" t="s">
+        <v>165</v>
+      </c>
+      <c r="F63" s="11" t="s">
+        <v>168</v>
+      </c>
+      <c r="G63" s="11" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="64" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A64" s="12">
+        <v>383002</v>
+      </c>
+      <c r="B64" s="7"/>
+      <c r="C64" s="7"/>
+      <c r="D64" s="11" t="s">
+        <v>160</v>
+      </c>
+      <c r="E64" s="11" t="s">
+        <v>165</v>
+      </c>
+      <c r="F64" s="11" t="s">
+        <v>168</v>
+      </c>
+      <c r="G64" s="11" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="65" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A65" s="12">
+        <v>383010</v>
+      </c>
+      <c r="B65" s="7"/>
+      <c r="C65" s="7"/>
+      <c r="D65" s="11" t="s">
+        <v>160</v>
+      </c>
+      <c r="E65" s="11" t="s">
+        <v>165</v>
+      </c>
+      <c r="F65" s="11" t="s">
+        <v>168</v>
+      </c>
+      <c r="G65" s="11" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="66" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A66" s="12">
+        <v>382330</v>
+      </c>
+      <c r="B66" s="7"/>
+      <c r="C66" s="7"/>
+      <c r="D66" s="11" t="s">
+        <v>161</v>
+      </c>
+      <c r="E66" s="11" t="s">
+        <v>165</v>
+      </c>
+      <c r="F66" s="11" t="s">
+        <v>171</v>
+      </c>
+      <c r="G66" s="11" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="67" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A67" s="12">
+        <v>382340</v>
+      </c>
+      <c r="B67" s="7"/>
+      <c r="C67" s="7"/>
+      <c r="D67" s="11" t="s">
+        <v>161</v>
+      </c>
+      <c r="E67" s="11" t="s">
+        <v>165</v>
+      </c>
+      <c r="F67" s="11" t="s">
+        <v>171</v>
+      </c>
+      <c r="G67" s="11" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="68" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A68" s="12">
+        <v>382345</v>
+      </c>
+      <c r="B68" s="7"/>
+      <c r="C68" s="7"/>
+      <c r="D68" s="11" t="s">
+        <v>161</v>
+      </c>
+      <c r="E68" s="11" t="s">
+        <v>165</v>
+      </c>
+      <c r="F68" s="11" t="s">
+        <v>171</v>
+      </c>
+      <c r="G68" s="11" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="69" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A69" s="12">
+        <v>382350</v>
+      </c>
+      <c r="B69" s="7"/>
+      <c r="C69" s="7"/>
+      <c r="D69" s="11" t="s">
+        <v>161</v>
+      </c>
+      <c r="E69" s="11" t="s">
+        <v>165</v>
+      </c>
+      <c r="F69" s="11" t="s">
+        <v>171</v>
+      </c>
+      <c r="G69" s="11" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="70" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A70" s="12">
+        <v>382440</v>
+      </c>
+      <c r="B70" s="7"/>
+      <c r="C70" s="7"/>
+      <c r="D70" s="11" t="s">
+        <v>161</v>
+      </c>
+      <c r="E70" s="11" t="s">
+        <v>165</v>
+      </c>
+      <c r="F70" s="11" t="s">
+        <v>171</v>
+      </c>
+      <c r="G70" s="11" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="71" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A71" s="12">
+        <v>382443</v>
+      </c>
+      <c r="B71" s="7"/>
+      <c r="C71" s="7"/>
+      <c r="D71" s="11" t="s">
+        <v>161</v>
+      </c>
+      <c r="E71" s="11" t="s">
+        <v>165</v>
+      </c>
+      <c r="F71" s="11" t="s">
+        <v>171</v>
+      </c>
+      <c r="G71" s="11" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="72" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A72" s="12">
+        <v>382445</v>
+      </c>
+      <c r="B72" s="7"/>
+      <c r="C72" s="7"/>
+      <c r="D72" s="11" t="s">
+        <v>161</v>
+      </c>
+      <c r="E72" s="11" t="s">
+        <v>165</v>
+      </c>
+      <c r="F72" s="11" t="s">
+        <v>171</v>
+      </c>
+      <c r="G72" s="11" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="73" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A73" s="12">
+        <v>387001</v>
+      </c>
+      <c r="B73" s="7"/>
+      <c r="C73" s="7"/>
+      <c r="D73" s="11" t="s">
+        <v>162</v>
+      </c>
+      <c r="E73" s="11" t="s">
+        <v>165</v>
+      </c>
+      <c r="F73" s="11" t="s">
+        <v>178</v>
+      </c>
+      <c r="G73" s="11" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="74" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A74" s="12">
+        <v>387002</v>
+      </c>
+      <c r="B74" s="7"/>
+      <c r="C74" s="7"/>
+      <c r="D74" s="11" t="s">
+        <v>162</v>
+      </c>
+      <c r="E74" s="11" t="s">
+        <v>165</v>
+      </c>
+      <c r="F74" s="11" t="s">
+        <v>178</v>
+      </c>
+      <c r="G74" s="11" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="75" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A75" s="12">
+        <v>387003</v>
+      </c>
+      <c r="B75" s="7"/>
+      <c r="C75" s="7"/>
+      <c r="D75" s="11" t="s">
+        <v>162</v>
+      </c>
+      <c r="E75" s="11" t="s">
+        <v>165</v>
+      </c>
+      <c r="F75" s="11" t="s">
+        <v>178</v>
+      </c>
+      <c r="G75" s="11" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="76" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A76" s="12">
+        <v>387004</v>
+      </c>
+      <c r="B76" s="7"/>
+      <c r="C76" s="7"/>
+      <c r="D76" s="11" t="s">
+        <v>162</v>
+      </c>
+      <c r="E76" s="11" t="s">
+        <v>165</v>
+      </c>
+      <c r="F76" s="11" t="s">
+        <v>178</v>
+      </c>
+      <c r="G76" s="11" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="77" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A77" s="12">
+        <v>387005</v>
+      </c>
+      <c r="B77" s="7"/>
+      <c r="C77" s="7"/>
+      <c r="D77" s="11" t="s">
+        <v>162</v>
+      </c>
+      <c r="E77" s="11" t="s">
+        <v>165</v>
+      </c>
+      <c r="F77" s="11" t="s">
+        <v>178</v>
+      </c>
+      <c r="G77" s="11" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="78" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A78" s="12">
+        <v>387006</v>
+      </c>
+      <c r="B78" s="7"/>
+      <c r="C78" s="7"/>
+      <c r="D78" s="11" t="s">
+        <v>162</v>
+      </c>
+      <c r="E78" s="11" t="s">
+        <v>165</v>
+      </c>
+      <c r="F78" s="11" t="s">
+        <v>178</v>
+      </c>
+      <c r="G78" s="11" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="79" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A79" s="12">
+        <v>390001</v>
+      </c>
+      <c r="B79" s="7"/>
+      <c r="C79" s="7"/>
+      <c r="D79" s="11" t="s">
+        <v>163</v>
+      </c>
+      <c r="E79" s="11" t="s">
+        <v>165</v>
+      </c>
+      <c r="F79" s="11" t="s">
+        <v>179</v>
+      </c>
+      <c r="G79" s="11" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="80" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A80" s="12">
+        <v>390002</v>
+      </c>
+      <c r="B80" s="7"/>
+      <c r="C80" s="7"/>
+      <c r="D80" s="11" t="s">
+        <v>163</v>
+      </c>
+      <c r="E80" s="11" t="s">
+        <v>165</v>
+      </c>
+      <c r="F80" s="11" t="s">
+        <v>179</v>
+      </c>
+      <c r="G80" s="11" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="81" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A81" s="12">
+        <v>390003</v>
+      </c>
+      <c r="B81" s="7"/>
+      <c r="C81" s="7"/>
+      <c r="D81" s="11" t="s">
+        <v>163</v>
+      </c>
+      <c r="E81" s="11" t="s">
+        <v>165</v>
+      </c>
+      <c r="F81" s="11" t="s">
+        <v>179</v>
+      </c>
+      <c r="G81" s="11" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="82" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A82" s="12">
+        <v>390004</v>
+      </c>
+      <c r="B82" s="7"/>
+      <c r="C82" s="7"/>
+      <c r="D82" s="11" t="s">
+        <v>163</v>
+      </c>
+      <c r="E82" s="11" t="s">
+        <v>165</v>
+      </c>
+      <c r="F82" s="11" t="s">
+        <v>179</v>
+      </c>
+      <c r="G82" s="11" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="83" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A83" s="12">
+        <v>390005</v>
+      </c>
+      <c r="B83" s="7"/>
+      <c r="C83" s="7"/>
+      <c r="D83" s="11" t="s">
+        <v>163</v>
+      </c>
+      <c r="E83" s="11" t="s">
+        <v>165</v>
+      </c>
+      <c r="F83" s="11" t="s">
+        <v>179</v>
+      </c>
+      <c r="G83" s="11" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="84" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A84" s="12">
+        <v>390006</v>
+      </c>
+      <c r="B84" s="7"/>
+      <c r="C84" s="7"/>
+      <c r="D84" s="11" t="s">
+        <v>163</v>
+      </c>
+      <c r="E84" s="11" t="s">
+        <v>165</v>
+      </c>
+      <c r="F84" s="11" t="s">
+        <v>179</v>
+      </c>
+      <c r="G84" s="11" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="85" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A85" s="12">
+        <v>390007</v>
+      </c>
+      <c r="B85" s="7"/>
+      <c r="C85" s="7"/>
+      <c r="D85" s="11" t="s">
+        <v>163</v>
+      </c>
+      <c r="E85" s="11" t="s">
+        <v>165</v>
+      </c>
+      <c r="F85" s="11" t="s">
+        <v>179</v>
+      </c>
+      <c r="G85" s="11" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="86" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A86" s="12">
+        <v>390008</v>
+      </c>
+      <c r="B86" s="7"/>
+      <c r="C86" s="7"/>
+      <c r="D86" s="11" t="s">
+        <v>163</v>
+      </c>
+      <c r="E86" s="11" t="s">
+        <v>165</v>
+      </c>
+      <c r="F86" s="11" t="s">
+        <v>179</v>
+      </c>
+      <c r="G86" s="11" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="87" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A87" s="12">
+        <v>390009</v>
+      </c>
+      <c r="B87" s="7"/>
+      <c r="C87" s="7"/>
+      <c r="D87" s="11" t="s">
+        <v>163</v>
+      </c>
+      <c r="E87" s="11" t="s">
+        <v>165</v>
+      </c>
+      <c r="F87" s="11" t="s">
+        <v>179</v>
+      </c>
+      <c r="G87" s="11" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="88" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A88" s="12">
+        <v>390010</v>
+      </c>
+      <c r="B88" s="7"/>
+      <c r="C88" s="7"/>
+      <c r="D88" s="11" t="s">
+        <v>163</v>
+      </c>
+      <c r="E88" s="11" t="s">
+        <v>165</v>
+      </c>
+      <c r="F88" s="11" t="s">
+        <v>179</v>
+      </c>
+      <c r="G88" s="11" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="89" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A89" s="12">
+        <v>390011</v>
+      </c>
+      <c r="B89" s="7"/>
+      <c r="C89" s="7"/>
+      <c r="D89" s="11" t="s">
+        <v>163</v>
+      </c>
+      <c r="E89" s="11" t="s">
+        <v>165</v>
+      </c>
+      <c r="F89" s="11" t="s">
+        <v>179</v>
+      </c>
+      <c r="G89" s="11" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="90" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A90" s="12">
+        <v>390012</v>
+      </c>
+      <c r="B90" s="7"/>
+      <c r="C90" s="7"/>
+      <c r="D90" s="11" t="s">
+        <v>163</v>
+      </c>
+      <c r="E90" s="11" t="s">
+        <v>165</v>
+      </c>
+      <c r="F90" s="11" t="s">
+        <v>179</v>
+      </c>
+      <c r="G90" s="11" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="91" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A91" s="12">
+        <v>390013</v>
+      </c>
+      <c r="B91" s="7"/>
+      <c r="C91" s="7"/>
+      <c r="D91" s="11" t="s">
+        <v>163</v>
+      </c>
+      <c r="E91" s="11" t="s">
+        <v>165</v>
+      </c>
+      <c r="F91" s="11" t="s">
+        <v>179</v>
+      </c>
+      <c r="G91" s="11" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="92" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A92" s="12">
+        <v>390014</v>
+      </c>
+      <c r="B92" s="7"/>
+      <c r="C92" s="7"/>
+      <c r="D92" s="11" t="s">
+        <v>163</v>
+      </c>
+      <c r="E92" s="11" t="s">
+        <v>165</v>
+      </c>
+      <c r="F92" s="11" t="s">
+        <v>179</v>
+      </c>
+      <c r="G92" s="11" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="93" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A93" s="12">
+        <v>390015</v>
+      </c>
+      <c r="B93" s="7"/>
+      <c r="C93" s="7"/>
+      <c r="D93" s="11" t="s">
+        <v>163</v>
+      </c>
+      <c r="E93" s="11" t="s">
+        <v>165</v>
+      </c>
+      <c r="F93" s="11" t="s">
+        <v>179</v>
+      </c>
+      <c r="G93" s="11" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="94" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A94" s="12">
+        <v>390016</v>
+      </c>
+      <c r="B94" s="7"/>
+      <c r="C94" s="7"/>
+      <c r="D94" s="11" t="s">
+        <v>163</v>
+      </c>
+      <c r="E94" s="11" t="s">
+        <v>165</v>
+      </c>
+      <c r="F94" s="11" t="s">
+        <v>179</v>
+      </c>
+      <c r="G94" s="11" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="95" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A95" s="12">
+        <v>390017</v>
+      </c>
+      <c r="B95" s="7"/>
+      <c r="C95" s="7"/>
+      <c r="D95" s="11" t="s">
+        <v>163</v>
+      </c>
+      <c r="E95" s="11" t="s">
+        <v>165</v>
+      </c>
+      <c r="F95" s="11" t="s">
+        <v>179</v>
+      </c>
+      <c r="G95" s="11" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="96" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A96" s="12">
+        <v>390018</v>
+      </c>
+      <c r="B96" s="7"/>
+      <c r="C96" s="7"/>
+      <c r="D96" s="11" t="s">
+        <v>163</v>
+      </c>
+      <c r="E96" s="11" t="s">
+        <v>165</v>
+      </c>
+      <c r="F96" s="11" t="s">
+        <v>179</v>
+      </c>
+      <c r="G96" s="11" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="97" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A97" s="12">
+        <v>390019</v>
+      </c>
+      <c r="B97" s="7"/>
+      <c r="C97" s="7"/>
+      <c r="D97" s="11" t="s">
+        <v>163</v>
+      </c>
+      <c r="E97" s="11" t="s">
+        <v>165</v>
+      </c>
+      <c r="F97" s="11" t="s">
+        <v>179</v>
+      </c>
+      <c r="G97" s="11" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="98" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A98" s="12">
+        <v>390020</v>
+      </c>
+      <c r="B98" s="7"/>
+      <c r="C98" s="7"/>
+      <c r="D98" s="11" t="s">
+        <v>163</v>
+      </c>
+      <c r="E98" s="11" t="s">
+        <v>165</v>
+      </c>
+      <c r="F98" s="11" t="s">
+        <v>179</v>
+      </c>
+      <c r="G98" s="11" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="99" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A99" s="12">
+        <v>390021</v>
+      </c>
+      <c r="B99" s="7"/>
+      <c r="C99" s="7"/>
+      <c r="D99" s="11" t="s">
+        <v>163</v>
+      </c>
+      <c r="E99" s="11" t="s">
+        <v>165</v>
+      </c>
+      <c r="F99" s="11" t="s">
+        <v>179</v>
+      </c>
+      <c r="G99" s="11" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="100" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A100" s="12">
+        <v>390022</v>
+      </c>
+      <c r="B100" s="7"/>
+      <c r="C100" s="7"/>
+      <c r="D100" s="11" t="s">
+        <v>163</v>
+      </c>
+      <c r="E100" s="11" t="s">
+        <v>165</v>
+      </c>
+      <c r="F100" s="11" t="s">
+        <v>179</v>
+      </c>
+      <c r="G100" s="11" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="101" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A101" s="12">
+        <v>390023</v>
+      </c>
+      <c r="B101" s="7"/>
+      <c r="C101" s="7"/>
+      <c r="D101" s="11" t="s">
+        <v>163</v>
+      </c>
+      <c r="E101" s="11" t="s">
+        <v>165</v>
+      </c>
+      <c r="F101" s="11" t="s">
+        <v>179</v>
+      </c>
+      <c r="G101" s="11" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="102" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A102" s="12">
+        <v>390024</v>
+      </c>
+      <c r="B102" s="7"/>
+      <c r="C102" s="7"/>
+      <c r="D102" s="11" t="s">
+        <v>163</v>
+      </c>
+      <c r="E102" s="11" t="s">
+        <v>165</v>
+      </c>
+      <c r="F102" s="11" t="s">
+        <v>179</v>
+      </c>
+      <c r="G102" s="11" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="103" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A103" s="12">
+        <v>390025</v>
+      </c>
+      <c r="B103" s="7"/>
+      <c r="C103" s="7"/>
+      <c r="D103" s="11" t="s">
+        <v>163</v>
+      </c>
+      <c r="E103" s="11" t="s">
+        <v>165</v>
+      </c>
+      <c r="F103" s="11" t="s">
+        <v>179</v>
+      </c>
+      <c r="G103" s="11" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="104" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A104" s="12">
+        <v>390026</v>
+      </c>
+      <c r="B104" s="7"/>
+      <c r="C104" s="7"/>
+      <c r="D104" s="11" t="s">
+        <v>163</v>
+      </c>
+      <c r="E104" s="11" t="s">
+        <v>165</v>
+      </c>
+      <c r="F104" s="11" t="s">
+        <v>179</v>
+      </c>
+      <c r="G104" s="11" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="105" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A105" s="12">
+        <v>390027</v>
+      </c>
+      <c r="B105" s="7"/>
+      <c r="C105" s="7"/>
+      <c r="D105" s="11" t="s">
+        <v>163</v>
+      </c>
+      <c r="E105" s="11" t="s">
+        <v>165</v>
+      </c>
+      <c r="F105" s="11" t="s">
+        <v>179</v>
+      </c>
+      <c r="G105" s="11" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="106" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A106" s="12">
+        <v>390028</v>
+      </c>
+      <c r="B106" s="7"/>
+      <c r="C106" s="7"/>
+      <c r="D106" s="11" t="s">
+        <v>163</v>
+      </c>
+      <c r="E106" s="11" t="s">
+        <v>165</v>
+      </c>
+      <c r="F106" s="11" t="s">
+        <v>179</v>
+      </c>
+      <c r="G106" s="11" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="107" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A107" s="12">
+        <v>390029</v>
+      </c>
+      <c r="B107" s="7"/>
+      <c r="C107" s="7"/>
+      <c r="D107" s="11" t="s">
+        <v>163</v>
+      </c>
+      <c r="E107" s="11" t="s">
+        <v>165</v>
+      </c>
+      <c r="F107" s="11" t="s">
+        <v>179</v>
+      </c>
+      <c r="G107" s="11" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="108" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A108" s="12">
+        <v>390030</v>
+      </c>
+      <c r="B108" s="7"/>
+      <c r="C108" s="7"/>
+      <c r="D108" s="11" t="s">
+        <v>163</v>
+      </c>
+      <c r="E108" s="11" t="s">
+        <v>165</v>
+      </c>
+      <c r="F108" s="11" t="s">
+        <v>179</v>
+      </c>
+      <c r="G108" s="11" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="109" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A109" s="12">
+        <v>390031</v>
+      </c>
+      <c r="B109" s="7"/>
+      <c r="C109" s="7"/>
+      <c r="D109" s="11" t="s">
+        <v>163</v>
+      </c>
+      <c r="E109" s="11" t="s">
+        <v>165</v>
+      </c>
+      <c r="F109" s="11" t="s">
+        <v>179</v>
+      </c>
+      <c r="G109" s="11" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="110" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A110" s="12">
+        <v>390032</v>
+      </c>
+      <c r="B110" s="7"/>
+      <c r="C110" s="7"/>
+      <c r="D110" s="11" t="s">
+        <v>163</v>
+      </c>
+      <c r="E110" s="11" t="s">
+        <v>165</v>
+      </c>
+      <c r="F110" s="11" t="s">
+        <v>179</v>
+      </c>
+      <c r="G110" s="11" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="111" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A111" s="12">
+        <v>389001</v>
+      </c>
+      <c r="B111" s="7"/>
+      <c r="C111" s="7"/>
+      <c r="D111" s="11" t="s">
+        <v>164</v>
+      </c>
+      <c r="E111" s="11" t="s">
+        <v>165</v>
+      </c>
+      <c r="F111" s="11" t="s">
+        <v>180</v>
+      </c>
+      <c r="G111" s="11" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="112" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A112" s="13">
+        <v>389002</v>
+      </c>
+      <c r="B112" s="14"/>
+      <c r="C112" s="14"/>
+      <c r="D112" s="11" t="s">
+        <v>164</v>
+      </c>
+      <c r="E112" s="11" t="s">
+        <v>165</v>
+      </c>
+      <c r="F112" s="11" t="s">
+        <v>180</v>
+      </c>
+      <c r="G112" s="11" t="s">
+        <v>181</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">

</xml_diff>

<commit_message>
Load PINs added to the sheet without coordinates, and add two of them
A row with no latitude or longitude was skipped without a word, so the
two PINs added to the locations sheet (160055 Mohali, 383205 Prantij)
never reached the server. Such a row is now placed from its PIN code and
checked against its state, and any row that still cannot be loaded is
reported after the sync instead of vanishing.

The sync message also read totals the API never sends, and showed
"undefined"; it now shows the real ones.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Geocoded_Ad_Targeting_Locations_FINAL.xlsx
+++ b/Geocoded_Ad_Targeting_Locations_FINAL.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP\Downloads\G-Map_Data_Scraper_2.0\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8FF92AC9-4AE1-422F-8976-13A7F4FF7345}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{25367C65-9D59-4FFF-87B1-22B5894095AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{2EFE7CA6-FAD9-449D-9EE4-AAC15D71DE5D}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="507" uniqueCount="182">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="515" uniqueCount="185">
   <si>
     <t>PIN Code</t>
   </si>
@@ -571,6 +571,15 @@
   </si>
   <si>
     <t>Bhuravav/Godhra</t>
+  </si>
+  <si>
+    <t>Prantij</t>
+  </si>
+  <si>
+    <t>MOHALI</t>
+  </si>
+  <si>
+    <t>Sahibzada Ajit Singh Nagar</t>
   </si>
 </sst>
 </file>
@@ -608,7 +617,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -648,6 +657,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="4" tint="-0.249977111117893"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -692,7 +707,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -728,6 +743,12 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -927,8 +948,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{40D995E3-44C6-468A-840D-F24E2D0786F7}" name="Table1" displayName="Table1" ref="A1:G112" totalsRowShown="0" headerRowDxfId="7">
-  <autoFilter ref="A1:G112" xr:uid="{40D995E3-44C6-468A-840D-F24E2D0786F7}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{40D995E3-44C6-468A-840D-F24E2D0786F7}" name="Table1" displayName="Table1" ref="A1:G114" totalsRowShown="0" headerRowDxfId="7">
+  <autoFilter ref="A1:G114" xr:uid="{40D995E3-44C6-468A-840D-F24E2D0786F7}"/>
   <tableColumns count="7">
     <tableColumn id="1" xr3:uid="{6667905F-B31C-47BA-93E7-8506475DE500}" name="PIN Code" dataDxfId="6"/>
     <tableColumn id="2" xr3:uid="{755243FA-4E53-40DE-B529-B2791CD1B1FD}" name="Latitude" dataDxfId="5"/>
@@ -1239,7 +1260,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6B92FE42-A60B-4A3F-BBB0-B7F38A1791FE}">
-  <dimension ref="A1:G112"/>
+  <dimension ref="A1:G114"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="15.36328125" style="1" customWidth="1"/>
@@ -2425,60 +2446,56 @@
       </c>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A52" s="5" t="s">
-        <v>42</v>
-      </c>
-      <c r="B52" s="7">
-        <v>30.825246</v>
-      </c>
-      <c r="C52" s="7">
-        <v>76.177547500000003</v>
-      </c>
+      <c r="A52" s="16">
+        <v>160055</v>
+      </c>
+      <c r="B52" s="7"/>
+      <c r="C52" s="7"/>
       <c r="D52" s="7" t="s">
-        <v>117</v>
+        <v>183</v>
       </c>
       <c r="E52" s="7" t="s">
         <v>99</v>
       </c>
-      <c r="F52" s="7" t="s">
-        <v>121</v>
-      </c>
-      <c r="G52" s="7" t="s">
-        <v>121</v>
+      <c r="F52" t="s">
+        <v>184</v>
+      </c>
+      <c r="G52" t="s">
+        <v>184</v>
       </c>
     </row>
     <row r="53" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A53" s="5" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B53" s="7">
-        <v>29.9486566</v>
+        <v>30.825246</v>
       </c>
       <c r="C53" s="7">
-        <v>74.737280900000002</v>
+        <v>76.177547500000003</v>
       </c>
       <c r="D53" s="7" t="s">
-        <v>122</v>
+        <v>117</v>
       </c>
       <c r="E53" s="7" t="s">
-        <v>89</v>
+        <v>99</v>
       </c>
       <c r="F53" s="7" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="G53" s="7" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
     </row>
     <row r="54" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A54" s="5" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B54" s="7">
-        <v>29.444108</v>
+        <v>29.9486566</v>
       </c>
       <c r="C54" s="7">
-        <v>74.657949900000006</v>
+        <v>74.737280900000002</v>
       </c>
       <c r="D54" s="7" t="s">
         <v>122</v>
@@ -2487,21 +2504,21 @@
         <v>89</v>
       </c>
       <c r="F54" s="7" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="G54" s="7" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="55" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A55" s="5" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B55" s="7">
-        <v>29.5240902</v>
+        <v>29.444108</v>
       </c>
       <c r="C55" s="7">
-        <v>74.836932700000006</v>
+        <v>74.657949900000006</v>
       </c>
       <c r="D55" s="7" t="s">
         <v>122</v>
@@ -2510,21 +2527,21 @@
         <v>89</v>
       </c>
       <c r="F55" s="7" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="G55" s="7" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A56" s="5" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B56" s="7">
-        <v>29.5372849</v>
+        <v>29.5240902</v>
       </c>
       <c r="C56" s="7">
-        <v>75.037764899999999</v>
+        <v>74.836932700000006</v>
       </c>
       <c r="D56" s="7" t="s">
         <v>122</v>
@@ -2533,44 +2550,44 @@
         <v>89</v>
       </c>
       <c r="F56" s="7" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G56" s="7" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A57" s="5" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B57" s="7">
-        <v>30.3042628</v>
+        <v>29.5372849</v>
       </c>
       <c r="C57" s="7">
-        <v>77.302725300000006</v>
+        <v>75.037764899999999</v>
       </c>
       <c r="D57" s="7" t="s">
-        <v>127</v>
+        <v>122</v>
       </c>
       <c r="E57" s="7" t="s">
         <v>89</v>
       </c>
       <c r="F57" s="7" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="G57" s="7" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A58" s="5" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B58" s="7">
-        <v>30.245567999999999</v>
+        <v>30.3042628</v>
       </c>
       <c r="C58" s="7">
-        <v>77.359232399999996</v>
+        <v>77.302725300000006</v>
       </c>
       <c r="D58" s="7" t="s">
         <v>127</v>
@@ -2579,21 +2596,21 @@
         <v>89</v>
       </c>
       <c r="F58" s="7" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="G58" s="7" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A59" s="5" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B59" s="7">
-        <v>30.117322000000001</v>
+        <v>30.245567999999999</v>
       </c>
       <c r="C59" s="7">
-        <v>77.287663699999996</v>
+        <v>77.359232399999996</v>
       </c>
       <c r="D59" s="7" t="s">
         <v>127</v>
@@ -2602,34 +2619,38 @@
         <v>89</v>
       </c>
       <c r="F59" s="7" t="s">
+        <v>129</v>
+      </c>
+      <c r="G59" s="7" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="60" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A60" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="B60" s="7">
+        <v>30.117322000000001</v>
+      </c>
+      <c r="C60" s="7">
+        <v>77.287663699999996</v>
+      </c>
+      <c r="D60" s="7" t="s">
+        <v>127</v>
+      </c>
+      <c r="E60" s="7" t="s">
+        <v>89</v>
+      </c>
+      <c r="F60" s="7" t="s">
         <v>130</v>
       </c>
-      <c r="G59" s="7" t="s">
+      <c r="G60" s="7" t="s">
         <v>130</v>
-      </c>
-    </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A60" s="12">
-        <v>385001</v>
-      </c>
-      <c r="B60" s="7"/>
-      <c r="C60" s="7"/>
-      <c r="D60" s="11" t="s">
-        <v>159</v>
-      </c>
-      <c r="E60" s="11" t="s">
-        <v>165</v>
-      </c>
-      <c r="F60" s="11" t="s">
-        <v>166</v>
-      </c>
-      <c r="G60" s="11" t="s">
-        <v>166</v>
       </c>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A61" s="12">
-        <v>385002</v>
+        <v>385001</v>
       </c>
       <c r="B61" s="7"/>
       <c r="C61" s="7"/>
@@ -2643,12 +2664,12 @@
         <v>166</v>
       </c>
       <c r="G61" s="11" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A62" s="12">
-        <v>385010</v>
+        <v>385002</v>
       </c>
       <c r="B62" s="7"/>
       <c r="C62" s="7"/>
@@ -2667,26 +2688,26 @@
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A63" s="12">
-        <v>383001</v>
+        <v>385010</v>
       </c>
       <c r="B63" s="7"/>
       <c r="C63" s="7"/>
       <c r="D63" s="11" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="E63" s="11" t="s">
         <v>165</v>
       </c>
       <c r="F63" s="11" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="G63" s="11" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A64" s="12">
-        <v>383002</v>
+        <v>383001</v>
       </c>
       <c r="B64" s="7"/>
       <c r="C64" s="7"/>
@@ -2700,12 +2721,12 @@
         <v>168</v>
       </c>
       <c r="G64" s="11" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
     </row>
     <row r="65" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A65" s="12">
-        <v>383010</v>
+        <v>383002</v>
       </c>
       <c r="B65" s="7"/>
       <c r="C65" s="7"/>
@@ -2719,50 +2740,50 @@
         <v>168</v>
       </c>
       <c r="G65" s="11" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="66" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A66" s="12">
-        <v>382330</v>
+      <c r="A66" s="15">
+        <v>383205</v>
       </c>
       <c r="B66" s="7"/>
       <c r="C66" s="7"/>
       <c r="D66" s="11" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="E66" s="11" t="s">
         <v>165</v>
       </c>
-      <c r="F66" s="11" t="s">
-        <v>171</v>
-      </c>
-      <c r="G66" s="11" t="s">
-        <v>172</v>
+      <c r="F66" t="s">
+        <v>182</v>
+      </c>
+      <c r="G66" t="s">
+        <v>182</v>
       </c>
     </row>
     <row r="67" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A67" s="12">
-        <v>382340</v>
+        <v>383010</v>
       </c>
       <c r="B67" s="7"/>
       <c r="C67" s="7"/>
       <c r="D67" s="11" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="E67" s="11" t="s">
         <v>165</v>
       </c>
       <c r="F67" s="11" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="G67" s="11" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
     </row>
     <row r="68" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A68" s="12">
-        <v>382345</v>
+        <v>382330</v>
       </c>
       <c r="B68" s="7"/>
       <c r="C68" s="7"/>
@@ -2776,12 +2797,12 @@
         <v>171</v>
       </c>
       <c r="G68" s="11" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
     </row>
     <row r="69" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A69" s="12">
-        <v>382350</v>
+        <v>382340</v>
       </c>
       <c r="B69" s="7"/>
       <c r="C69" s="7"/>
@@ -2795,12 +2816,12 @@
         <v>171</v>
       </c>
       <c r="G69" s="11" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
     </row>
     <row r="70" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A70" s="12">
-        <v>382440</v>
+        <v>382345</v>
       </c>
       <c r="B70" s="7"/>
       <c r="C70" s="7"/>
@@ -2814,12 +2835,12 @@
         <v>171</v>
       </c>
       <c r="G70" s="11" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
     </row>
     <row r="71" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A71" s="12">
-        <v>382443</v>
+        <v>382350</v>
       </c>
       <c r="B71" s="7"/>
       <c r="C71" s="7"/>
@@ -2833,12 +2854,12 @@
         <v>171</v>
       </c>
       <c r="G71" s="11" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
     </row>
     <row r="72" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A72" s="12">
-        <v>382445</v>
+        <v>382440</v>
       </c>
       <c r="B72" s="7"/>
       <c r="C72" s="7"/>
@@ -2852,50 +2873,50 @@
         <v>171</v>
       </c>
       <c r="G72" s="11" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
     </row>
     <row r="73" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A73" s="12">
-        <v>387001</v>
+        <v>382443</v>
       </c>
       <c r="B73" s="7"/>
       <c r="C73" s="7"/>
       <c r="D73" s="11" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="E73" s="11" t="s">
         <v>165</v>
       </c>
       <c r="F73" s="11" t="s">
-        <v>178</v>
+        <v>171</v>
       </c>
       <c r="G73" s="11" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
     </row>
     <row r="74" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A74" s="12">
-        <v>387002</v>
+        <v>382445</v>
       </c>
       <c r="B74" s="7"/>
       <c r="C74" s="7"/>
       <c r="D74" s="11" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="E74" s="11" t="s">
         <v>165</v>
       </c>
       <c r="F74" s="11" t="s">
-        <v>178</v>
+        <v>171</v>
       </c>
       <c r="G74" s="11" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="75" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A75" s="12">
-        <v>387003</v>
+        <v>387001</v>
       </c>
       <c r="B75" s="7"/>
       <c r="C75" s="7"/>
@@ -2914,7 +2935,7 @@
     </row>
     <row r="76" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A76" s="12">
-        <v>387004</v>
+        <v>387002</v>
       </c>
       <c r="B76" s="7"/>
       <c r="C76" s="7"/>
@@ -2933,7 +2954,7 @@
     </row>
     <row r="77" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A77" s="12">
-        <v>387005</v>
+        <v>387003</v>
       </c>
       <c r="B77" s="7"/>
       <c r="C77" s="7"/>
@@ -2952,7 +2973,7 @@
     </row>
     <row r="78" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A78" s="12">
-        <v>387006</v>
+        <v>387004</v>
       </c>
       <c r="B78" s="7"/>
       <c r="C78" s="7"/>
@@ -2971,45 +2992,45 @@
     </row>
     <row r="79" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A79" s="12">
-        <v>390001</v>
+        <v>387005</v>
       </c>
       <c r="B79" s="7"/>
       <c r="C79" s="7"/>
       <c r="D79" s="11" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="E79" s="11" t="s">
         <v>165</v>
       </c>
       <c r="F79" s="11" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="G79" s="11" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="80" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A80" s="12">
-        <v>390002</v>
+        <v>387006</v>
       </c>
       <c r="B80" s="7"/>
       <c r="C80" s="7"/>
       <c r="D80" s="11" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="E80" s="11" t="s">
         <v>165</v>
       </c>
       <c r="F80" s="11" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="G80" s="11" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="81" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A81" s="12">
-        <v>390003</v>
+        <v>390001</v>
       </c>
       <c r="B81" s="7"/>
       <c r="C81" s="7"/>
@@ -3028,7 +3049,7 @@
     </row>
     <row r="82" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A82" s="12">
-        <v>390004</v>
+        <v>390002</v>
       </c>
       <c r="B82" s="7"/>
       <c r="C82" s="7"/>
@@ -3047,7 +3068,7 @@
     </row>
     <row r="83" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A83" s="12">
-        <v>390005</v>
+        <v>390003</v>
       </c>
       <c r="B83" s="7"/>
       <c r="C83" s="7"/>
@@ -3066,7 +3087,7 @@
     </row>
     <row r="84" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A84" s="12">
-        <v>390006</v>
+        <v>390004</v>
       </c>
       <c r="B84" s="7"/>
       <c r="C84" s="7"/>
@@ -3085,7 +3106,7 @@
     </row>
     <row r="85" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A85" s="12">
-        <v>390007</v>
+        <v>390005</v>
       </c>
       <c r="B85" s="7"/>
       <c r="C85" s="7"/>
@@ -3104,7 +3125,7 @@
     </row>
     <row r="86" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A86" s="12">
-        <v>390008</v>
+        <v>390006</v>
       </c>
       <c r="B86" s="7"/>
       <c r="C86" s="7"/>
@@ -3123,7 +3144,7 @@
     </row>
     <row r="87" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A87" s="12">
-        <v>390009</v>
+        <v>390007</v>
       </c>
       <c r="B87" s="7"/>
       <c r="C87" s="7"/>
@@ -3142,7 +3163,7 @@
     </row>
     <row r="88" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A88" s="12">
-        <v>390010</v>
+        <v>390008</v>
       </c>
       <c r="B88" s="7"/>
       <c r="C88" s="7"/>
@@ -3161,7 +3182,7 @@
     </row>
     <row r="89" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A89" s="12">
-        <v>390011</v>
+        <v>390009</v>
       </c>
       <c r="B89" s="7"/>
       <c r="C89" s="7"/>
@@ -3180,7 +3201,7 @@
     </row>
     <row r="90" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A90" s="12">
-        <v>390012</v>
+        <v>390010</v>
       </c>
       <c r="B90" s="7"/>
       <c r="C90" s="7"/>
@@ -3199,7 +3220,7 @@
     </row>
     <row r="91" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A91" s="12">
-        <v>390013</v>
+        <v>390011</v>
       </c>
       <c r="B91" s="7"/>
       <c r="C91" s="7"/>
@@ -3218,7 +3239,7 @@
     </row>
     <row r="92" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A92" s="12">
-        <v>390014</v>
+        <v>390012</v>
       </c>
       <c r="B92" s="7"/>
       <c r="C92" s="7"/>
@@ -3237,7 +3258,7 @@
     </row>
     <row r="93" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A93" s="12">
-        <v>390015</v>
+        <v>390013</v>
       </c>
       <c r="B93" s="7"/>
       <c r="C93" s="7"/>
@@ -3256,7 +3277,7 @@
     </row>
     <row r="94" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A94" s="12">
-        <v>390016</v>
+        <v>390014</v>
       </c>
       <c r="B94" s="7"/>
       <c r="C94" s="7"/>
@@ -3275,7 +3296,7 @@
     </row>
     <row r="95" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A95" s="12">
-        <v>390017</v>
+        <v>390015</v>
       </c>
       <c r="B95" s="7"/>
       <c r="C95" s="7"/>
@@ -3294,7 +3315,7 @@
     </row>
     <row r="96" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A96" s="12">
-        <v>390018</v>
+        <v>390016</v>
       </c>
       <c r="B96" s="7"/>
       <c r="C96" s="7"/>
@@ -3313,7 +3334,7 @@
     </row>
     <row r="97" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A97" s="12">
-        <v>390019</v>
+        <v>390017</v>
       </c>
       <c r="B97" s="7"/>
       <c r="C97" s="7"/>
@@ -3332,7 +3353,7 @@
     </row>
     <row r="98" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A98" s="12">
-        <v>390020</v>
+        <v>390018</v>
       </c>
       <c r="B98" s="7"/>
       <c r="C98" s="7"/>
@@ -3351,7 +3372,7 @@
     </row>
     <row r="99" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A99" s="12">
-        <v>390021</v>
+        <v>390019</v>
       </c>
       <c r="B99" s="7"/>
       <c r="C99" s="7"/>
@@ -3370,7 +3391,7 @@
     </row>
     <row r="100" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A100" s="12">
-        <v>390022</v>
+        <v>390020</v>
       </c>
       <c r="B100" s="7"/>
       <c r="C100" s="7"/>
@@ -3389,7 +3410,7 @@
     </row>
     <row r="101" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A101" s="12">
-        <v>390023</v>
+        <v>390021</v>
       </c>
       <c r="B101" s="7"/>
       <c r="C101" s="7"/>
@@ -3408,7 +3429,7 @@
     </row>
     <row r="102" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A102" s="12">
-        <v>390024</v>
+        <v>390022</v>
       </c>
       <c r="B102" s="7"/>
       <c r="C102" s="7"/>
@@ -3427,7 +3448,7 @@
     </row>
     <row r="103" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A103" s="12">
-        <v>390025</v>
+        <v>390023</v>
       </c>
       <c r="B103" s="7"/>
       <c r="C103" s="7"/>
@@ -3446,7 +3467,7 @@
     </row>
     <row r="104" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A104" s="12">
-        <v>390026</v>
+        <v>390024</v>
       </c>
       <c r="B104" s="7"/>
       <c r="C104" s="7"/>
@@ -3465,7 +3486,7 @@
     </row>
     <row r="105" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A105" s="12">
-        <v>390027</v>
+        <v>390025</v>
       </c>
       <c r="B105" s="7"/>
       <c r="C105" s="7"/>
@@ -3484,7 +3505,7 @@
     </row>
     <row r="106" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A106" s="12">
-        <v>390028</v>
+        <v>390026</v>
       </c>
       <c r="B106" s="7"/>
       <c r="C106" s="7"/>
@@ -3503,7 +3524,7 @@
     </row>
     <row r="107" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A107" s="12">
-        <v>390029</v>
+        <v>390027</v>
       </c>
       <c r="B107" s="7"/>
       <c r="C107" s="7"/>
@@ -3522,7 +3543,7 @@
     </row>
     <row r="108" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A108" s="12">
-        <v>390030</v>
+        <v>390028</v>
       </c>
       <c r="B108" s="7"/>
       <c r="C108" s="7"/>
@@ -3541,7 +3562,7 @@
     </row>
     <row r="109" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A109" s="12">
-        <v>390031</v>
+        <v>390029</v>
       </c>
       <c r="B109" s="7"/>
       <c r="C109" s="7"/>
@@ -3560,7 +3581,7 @@
     </row>
     <row r="110" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A110" s="12">
-        <v>390032</v>
+        <v>390030</v>
       </c>
       <c r="B110" s="7"/>
       <c r="C110" s="7"/>
@@ -3579,39 +3600,77 @@
     </row>
     <row r="111" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A111" s="12">
-        <v>389001</v>
+        <v>390031</v>
       </c>
       <c r="B111" s="7"/>
       <c r="C111" s="7"/>
       <c r="D111" s="11" t="s">
+        <v>163</v>
+      </c>
+      <c r="E111" s="11" t="s">
+        <v>165</v>
+      </c>
+      <c r="F111" s="11" t="s">
+        <v>179</v>
+      </c>
+      <c r="G111" s="11" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="112" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A112" s="12">
+        <v>390032</v>
+      </c>
+      <c r="B112" s="7"/>
+      <c r="C112" s="7"/>
+      <c r="D112" s="11" t="s">
+        <v>163</v>
+      </c>
+      <c r="E112" s="11" t="s">
+        <v>165</v>
+      </c>
+      <c r="F112" s="11" t="s">
+        <v>179</v>
+      </c>
+      <c r="G112" s="11" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="113" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A113" s="12">
+        <v>389001</v>
+      </c>
+      <c r="B113" s="7"/>
+      <c r="C113" s="7"/>
+      <c r="D113" s="11" t="s">
         <v>164</v>
       </c>
-      <c r="E111" s="11" t="s">
-        <v>165</v>
-      </c>
-      <c r="F111" s="11" t="s">
+      <c r="E113" s="11" t="s">
+        <v>165</v>
+      </c>
+      <c r="F113" s="11" t="s">
         <v>180</v>
       </c>
-      <c r="G111" s="11" t="s">
+      <c r="G113" s="11" t="s">
         <v>180</v>
       </c>
     </row>
-    <row r="112" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A112" s="13">
+    <row r="114" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A114" s="13">
         <v>389002</v>
       </c>
-      <c r="B112" s="14"/>
-      <c r="C112" s="14"/>
-      <c r="D112" s="11" t="s">
+      <c r="B114" s="14"/>
+      <c r="C114" s="14"/>
+      <c r="D114" s="11" t="s">
         <v>164</v>
       </c>
-      <c r="E112" s="11" t="s">
-        <v>165</v>
-      </c>
-      <c r="F112" s="11" t="s">
+      <c r="E114" s="11" t="s">
+        <v>165</v>
+      </c>
+      <c r="F114" s="11" t="s">
         <v>180</v>
       </c>
-      <c r="G112" s="11" t="s">
+      <c r="G114" s="11" t="s">
         <v>181</v>
       </c>
     </row>

</xml_diff>